<commit_message>
FW trait data organization
</commit_message>
<xml_diff>
--- a/data_input/Data_dictionary_1_Database_field_descriptions.xlsx
+++ b/data_input/Data_dictionary_1_Database_field_descriptions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sync\R Workspace\Zooplankton_trait_database\data_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D96BD046-AA9E-4FC3-AA99-37FAD8092532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F475A5-00D0-4BBE-920F-4F73F0B56066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{BDC4C6F7-730B-4DDE-8FC0-ED27EE7DAC19}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{BDC4C6F7-730B-4DDE-8FC0-ED27EE7DAC19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="151">
   <si>
     <t>Field Name</t>
   </si>
@@ -544,9 +544,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -584,7 +584,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -690,7 +690,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -832,7 +832,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -840,7 +840,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9A15EA0-866A-4730-80F1-CCE293EE0F70}">
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="21.3984375" bestFit="1" customWidth="1"/>
@@ -949,24 +949,36 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -977,16 +989,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
@@ -997,16 +1009,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
         <v>9</v>
@@ -1017,16 +1029,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E10" t="s">
         <v>9</v>
@@ -1037,16 +1049,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
         <v>9</v>
@@ -1057,38 +1066,47 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
       </c>
       <c r="F13" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E14" t="s">
         <v>9</v>
@@ -1099,13 +1117,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>49</v>
+      </c>
+      <c r="D15" t="s">
+        <v>50</v>
       </c>
       <c r="E15" t="s">
         <v>9</v>
@@ -1116,16 +1137,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F16" t="s">
         <v>41</v>
@@ -1136,19 +1157,19 @@
         <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E17" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F17" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
@@ -1156,10 +1177,13 @@
         <v>47</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>57</v>
+      </c>
+      <c r="D18" t="s">
+        <v>58</v>
       </c>
       <c r="E18" t="s">
         <v>14</v>
@@ -1173,16 +1197,13 @@
         <v>47</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F19" t="s">
         <v>41</v>
@@ -1193,16 +1214,13 @@
         <v>47</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E20" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F20" t="s">
         <v>41</v>
@@ -1213,10 +1231,10 @@
         <v>47</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
@@ -1230,13 +1248,13 @@
         <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E22" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F22" t="s">
         <v>41</v>
@@ -1247,13 +1265,13 @@
         <v>47</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E23" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
         <v>41</v>
@@ -1264,10 +1282,10 @@
         <v>47</v>
       </c>
       <c r="B24" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C24" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E24" t="s">
         <v>14</v>
@@ -1281,13 +1299,13 @@
         <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E25" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F25" t="s">
         <v>41</v>
@@ -1298,16 +1316,19 @@
         <v>47</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>74</v>
+      </c>
+      <c r="D26" t="s">
+        <v>75</v>
       </c>
       <c r="E26" t="s">
         <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
@@ -1315,16 +1336,19 @@
         <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>77</v>
+      </c>
+      <c r="D27" t="s">
+        <v>78</v>
       </c>
       <c r="E27" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F27" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
@@ -1332,16 +1356,16 @@
         <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C28" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D28" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E28" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F28" t="s">
         <v>44</v>
@@ -1352,36 +1376,33 @@
         <v>47</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D29" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E29" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F29" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="C30" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D30" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E30" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F30" t="s">
         <v>44</v>
@@ -1389,19 +1410,22 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="B31" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C31" t="s">
-        <v>83</v>
+        <v>89</v>
+      </c>
+      <c r="D31" t="s">
+        <v>90</v>
       </c>
       <c r="E31" t="s">
         <v>9</v>
       </c>
       <c r="F31" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.45">
@@ -1409,19 +1433,19 @@
         <v>84</v>
       </c>
       <c r="B32" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="D32" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E32" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F32" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.45">
@@ -1429,19 +1453,19 @@
         <v>84</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C33" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D33" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E33" t="s">
         <v>9</v>
       </c>
       <c r="F33" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.45">
@@ -1449,13 +1473,13 @@
         <v>84</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C34" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D34" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E34" t="s">
         <v>9</v>
@@ -1469,19 +1493,19 @@
         <v>84</v>
       </c>
       <c r="B35" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C35" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="D35" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="E35" t="s">
         <v>9</v>
       </c>
       <c r="F35" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.45">
@@ -1489,19 +1513,19 @@
         <v>84</v>
       </c>
       <c r="B36" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C36" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D36" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E36" t="s">
         <v>9</v>
       </c>
       <c r="F36" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.45">
@@ -1509,13 +1533,13 @@
         <v>84</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C37" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D37" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E37" t="s">
         <v>9</v>
@@ -1529,13 +1553,13 @@
         <v>84</v>
       </c>
       <c r="B38" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C38" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="D38" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E38" t="s">
         <v>9</v>
@@ -1549,13 +1573,10 @@
         <v>84</v>
       </c>
       <c r="B39" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C39" t="s">
-        <v>107</v>
-      </c>
-      <c r="D39" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E39" t="s">
         <v>9</v>
@@ -1566,16 +1587,16 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="B40" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C40" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="D40" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E40" t="s">
         <v>9</v>
@@ -1586,13 +1607,16 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="B41" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C41" t="s">
-        <v>113</v>
+        <v>119</v>
+      </c>
+      <c r="D41" t="s">
+        <v>120</v>
       </c>
       <c r="E41" t="s">
         <v>9</v>
@@ -1606,19 +1630,19 @@
         <v>114</v>
       </c>
       <c r="B42" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C42" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D42" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="E42" t="s">
         <v>9</v>
       </c>
       <c r="F42" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.45">
@@ -1626,19 +1650,19 @@
         <v>114</v>
       </c>
       <c r="B43" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C43" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D43" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="E43" t="s">
         <v>9</v>
       </c>
       <c r="F43" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.45">
@@ -1646,13 +1670,13 @@
         <v>114</v>
       </c>
       <c r="B44" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C44" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D44" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E44" t="s">
         <v>9</v>
@@ -1666,13 +1690,13 @@
         <v>114</v>
       </c>
       <c r="B45" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C45" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D45" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="E45" t="s">
         <v>9</v>
@@ -1686,19 +1710,16 @@
         <v>114</v>
       </c>
       <c r="B46" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C46" t="s">
-        <v>128</v>
-      </c>
-      <c r="D46" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E46" t="s">
         <v>9</v>
       </c>
       <c r="F46" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.45">
@@ -1706,19 +1727,16 @@
         <v>114</v>
       </c>
       <c r="B47" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C47" t="s">
-        <v>131</v>
-      </c>
-      <c r="D47" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E47" t="s">
         <v>9</v>
       </c>
       <c r="F47" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.45">
@@ -1726,10 +1744,10 @@
         <v>114</v>
       </c>
       <c r="B48" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E48" t="s">
         <v>9</v>
@@ -1743,16 +1761,19 @@
         <v>114</v>
       </c>
       <c r="B49" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C49" t="s">
-        <v>136</v>
+        <v>140</v>
+      </c>
+      <c r="D49" t="s">
+        <v>141</v>
       </c>
       <c r="E49" t="s">
-        <v>9</v>
+        <v>142</v>
       </c>
       <c r="F49" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.45">
@@ -1760,16 +1781,16 @@
         <v>114</v>
       </c>
       <c r="B50" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C50" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E50" t="s">
-        <v>9</v>
+        <v>142</v>
       </c>
       <c r="F50" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.45">
@@ -1777,19 +1798,16 @@
         <v>114</v>
       </c>
       <c r="B51" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C51" t="s">
-        <v>140</v>
-      </c>
-      <c r="D51" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="E51" t="s">
-        <v>142</v>
+        <v>9</v>
       </c>
       <c r="F51" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.45">
@@ -1797,16 +1815,16 @@
         <v>114</v>
       </c>
       <c r="B52" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C52" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E52" t="s">
-        <v>142</v>
+        <v>14</v>
       </c>
       <c r="F52" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.45">
@@ -1814,49 +1832,15 @@
         <v>114</v>
       </c>
       <c r="B53" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C53" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E53" t="s">
         <v>9</v>
       </c>
       <c r="F53" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
-        <v>114</v>
-      </c>
-      <c r="B54" t="s">
-        <v>147</v>
-      </c>
-      <c r="C54" t="s">
-        <v>148</v>
-      </c>
-      <c r="E54" t="s">
-        <v>14</v>
-      </c>
-      <c r="F54" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
-        <v>114</v>
-      </c>
-      <c r="B55" t="s">
-        <v>149</v>
-      </c>
-      <c r="C55" t="s">
-        <v>150</v>
-      </c>
-      <c r="E55" t="s">
-        <v>9</v>
-      </c>
-      <c r="F55" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>